<commit_message>
feat(templates): coluna pagina web e internacionalizacao total dos modelos excel (PT, ES, EN, FR, PL)
</commit_message>
<xml_diff>
--- a/modelos_importacao/Modelo_Importacao_Clientes.xlsx
+++ b/modelos_importacao/Modelo_Importacao_Clientes.xlsx
@@ -397,23 +397,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:P5"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="36.83203125" customWidth="1"/>
+    <col min="3" max="3" width="36.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="34.83203125" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
     <col min="10" max="10" width="14.83203125" customWidth="1"/>
     <col min="11" max="11" width="18.83203125" customWidth="1"/>
     <col min="12" max="12" width="16.83203125" customWidth="1"/>
-    <col min="13" max="13" width="30.83203125" customWidth="1"/>
-    <col min="14" max="14" width="26.83203125" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="28.83203125" customWidth="1"/>
+    <col min="14" max="14" width="28.83203125" customWidth="1"/>
+    <col min="15" max="15" width="26.83203125" customWidth="1"/>
+    <col min="16" max="16" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -457,9 +458,12 @@
         <v>Email Geral</v>
       </c>
       <c r="N1" t="str">
+        <v>Página Web / Website</v>
+      </c>
+      <c r="O1" t="str">
         <v>Setor de Atividade</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Comercial Atribuído</v>
       </c>
     </row>
@@ -504,9 +508,12 @@
         <v>geral@dgadr.gov.pt</v>
       </c>
       <c r="N2" t="str">
+        <v>https://www.dgadr.gov.pt</v>
+      </c>
+      <c r="O2" t="str">
         <v>Administração Pública / Agricultura</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>José Centúrio</v>
       </c>
     </row>
@@ -515,25 +522,25 @@
         <v>Estatal</v>
       </c>
       <c r="B3" t="str">
-        <v>Ministério da Educação, Ciência e Inovação</v>
+        <v>Ministério da Saúde</v>
       </c>
       <c r="C3" t="str">
-        <v>Secretaria de Estado da Educação</v>
+        <v>Direção-Geral da Saúde</v>
       </c>
       <c r="D3" t="str">
         <v>500000456</v>
       </c>
       <c r="E3" t="str">
-        <v>Avenida 24 de Julho</v>
+        <v>Alameda Dom Afonso Henriques</v>
       </c>
       <c r="F3" t="str">
-        <v>140</v>
+        <v>45</v>
       </c>
       <c r="G3" t="str">
-        <v>4.º Andar</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>1399-025</v>
+        <v>1049-005</v>
       </c>
       <c r="I3" t="str">
         <v>Lisboa</v>
@@ -542,18 +549,21 @@
         <v>Portugal</v>
       </c>
       <c r="K3" t="str">
-        <v>+351 217 811 800</v>
+        <v>+351 218 430 500</v>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>961 000 000</v>
       </c>
       <c r="M3" t="str">
-        <v>gabinete.se@educacao.gov.pt</v>
+        <v>geral@dgs.min-saude.pt</v>
       </c>
       <c r="N3" t="str">
-        <v>Educação / Governo</v>
+        <v>https://www.dgs.pt</v>
       </c>
       <c r="O3" t="str">
+        <v>Saúde Pública / Governamental</v>
+      </c>
+      <c r="P3" t="str">
         <v>José Centúrio</v>
       </c>
     </row>
@@ -562,51 +572,104 @@
         <v>Privado</v>
       </c>
       <c r="B4" t="str">
-        <v>Mota-Engil, SGPS, S.A.</v>
+        <v>Galp Energia, SGPS, S.A.</v>
       </c>
       <c r="C4" t="str">
-        <v>Divisão de Logística e Infraestruturas</v>
+        <v/>
       </c>
       <c r="D4" t="str">
-        <v>502399694</v>
+        <v>504499777</v>
       </c>
       <c r="E4" t="str">
-        <v>Rua do Rego Lameiro</v>
+        <v>Rua Tomás da Fonseca, Torre A</v>
       </c>
       <c r="F4" t="str">
-        <v>38</v>
+        <v>Torre A</v>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>Piso 7</v>
       </c>
       <c r="H4" t="str">
-        <v>4300-454</v>
+        <v>1600-209</v>
       </c>
       <c r="I4" t="str">
-        <v>Porto</v>
+        <v>Lisboa</v>
       </c>
       <c r="J4" t="str">
         <v>Portugal</v>
       </c>
       <c r="K4" t="str">
-        <v>+351 225 190 300</v>
+        <v>+351 217 242 500</v>
       </c>
       <c r="L4" t="str">
-        <v>912 345 678</v>
+        <v>931 000 000</v>
       </c>
       <c r="M4" t="str">
-        <v>contacto@mota-engil.pt</v>
+        <v>comercial@galp.com</v>
       </c>
       <c r="N4" t="str">
-        <v>Construção e Logística</v>
+        <v>https://www.galp.com</v>
       </c>
       <c r="O4" t="str">
+        <v>Energia &amp; Combustíveis</v>
+      </c>
+      <c r="P4" t="str">
+        <v>José Centúrio</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Fundação</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Fundação Champalimaud</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Gabinete de Relações Externas</v>
+      </c>
+      <c r="D5" t="str">
+        <v>507000111</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Avenida Brasília</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>1400-038</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Lisboa</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Portugal</v>
+      </c>
+      <c r="K5" t="str">
+        <v>+351 210 480 200</v>
+      </c>
+      <c r="L5" t="str">
+        <v>925 000 000</v>
+      </c>
+      <c r="M5" t="str">
+        <v>info@fchampalimaud.org</v>
+      </c>
+      <c r="N5" t="str">
+        <v>https://fchampalimaud.org</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Investigação &amp; Saúde</v>
+      </c>
+      <c r="P5" t="str">
         <v>José Centúrio</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>